<commit_message>
Change repayment period for financed elec sector capital from 20 to 30 years
</commit_message>
<xml_diff>
--- a/InputData/elec/RPfFESCC/RPfFESCC Repayment Period for Financed Elec Sector Capital Costs.xlsx
+++ b/InputData/elec/RPfFESCC/RPfFESCC Repayment Period for Financed Elec Sector Capital Costs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\US\Models\eps-us\InputData\elec\RPfFESCC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\RPfFESCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80EC3107-A379-4815-A725-E40D4B74474C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6029335A-F32B-4B15-807C-3ED374EE4723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -457,17 +457,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="93" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -476,106 +476,106 @@
       </c>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B4" s="7">
         <v>2023</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B6" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>4</v>
       </c>
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B23" s="2"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B27" s="2"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
     </row>
@@ -594,13 +594,13 @@
     <tabColor theme="8" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="1" max="1" width="25.54296875" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>6</v>
       </c>
@@ -608,12 +608,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="3">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>